<commit_message>
Add USA500 cross-asset testing, update ranking system to v1.1
Strategy validated profitable on BOTH assets (GER40 + USA500):
- DEU.IDX-EUR: +1746% (Balanced), DD 8.0%, PF 2.72, WR 56.1%
- USA500.IDX-USD: +1451% (Balanced), DD 27.0%, PF 1.78, WR 61.1%

All walk-forward periods profitable on both assets (8/8).
Cross-asset score now properly computed across multiple assets.
Backtest engine uses adaptive thresholds (% of price) for multi-asset support.

https://claude.ai/code/session_018x91BkD24zVpNBh17M5GYw
</commit_message>
<xml_diff>
--- a/strategy_rankings.xlsx
+++ b/strategy_rankings.xlsx
@@ -447,14 +447,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA4"/>
+  <dimension ref="A1:AA7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="21" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="19" customWidth="1" min="8" max="8"/>
@@ -641,34 +641,34 @@
         </is>
       </c>
       <c r="F2" s="3" t="n">
-        <v>89.90000000000001</v>
+        <v>89.67</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>1691.36</v>
+        <v>1746.18</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>8</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>2.75</v>
+        <v>2.72</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>55.81</v>
+        <v>56.06</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>211.32</v>
+        <v>218.34</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>2.18</v>
+        <v>2.13</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>387</v>
+        <v>396</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>24.61</v>
+        <v>24.9</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>11.31</v>
+        <v>11.7</v>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
@@ -682,13 +682,13 @@
         <v>100</v>
       </c>
       <c r="S2" s="2" t="n">
-        <v>27</v>
+        <v>26.64</v>
       </c>
       <c r="T2" s="2" t="n">
         <v>25</v>
       </c>
       <c r="U2" s="2" t="n">
-        <v>12.91</v>
+        <v>13.03</v>
       </c>
       <c r="V2" s="2" t="n">
         <v>15</v>
@@ -708,7 +708,7 @@
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>2026-03-31 07:29</t>
+          <t>2026-03-31 07:47</t>
         </is>
       </c>
       <c r="AA2" s="2" t="inlineStr">
@@ -742,34 +742,34 @@
         </is>
       </c>
       <c r="F3" s="3" t="n">
-        <v>88.93000000000001</v>
+        <v>88.81999999999999</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>600.49</v>
+        <v>613.49</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>5.43</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>2.67</v>
+        <v>2.65</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>55.78</v>
+        <v>56.03</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>110.62</v>
+        <v>113.01</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>2.11</v>
+        <v>2.08</v>
       </c>
       <c r="M3" s="2" t="n">
-        <v>389</v>
+        <v>398</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>8.85</v>
+        <v>8.84</v>
       </c>
       <c r="O3" s="2" t="n">
-        <v>4.19</v>
+        <v>4.25</v>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
@@ -783,13 +783,13 @@
         <v>100</v>
       </c>
       <c r="S3" s="2" t="n">
-        <v>26.04</v>
+        <v>25.8</v>
       </c>
       <c r="T3" s="2" t="n">
         <v>25</v>
       </c>
       <c r="U3" s="2" t="n">
-        <v>12.89</v>
+        <v>13.02</v>
       </c>
       <c r="V3" s="2" t="n">
         <v>15</v>
@@ -809,7 +809,7 @@
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>2026-03-31 07:29</t>
+          <t>2026-03-31 07:47</t>
         </is>
       </c>
       <c r="AA3" s="2" t="inlineStr">
@@ -843,34 +843,34 @@
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>87.86</v>
+        <v>87.63</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>2828.28</v>
+        <v>2965.47</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>10.61</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>2.58</v>
+        <v>2.55</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>55.81</v>
+        <v>56.06</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>266.46</v>
+        <v>279.38</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>2.05</v>
+        <v>2</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>387</v>
+        <v>396</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>42.72</v>
+        <v>43.94</v>
       </c>
       <c r="O4" s="2" t="n">
-        <v>20.88</v>
+        <v>21.98</v>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
@@ -884,13 +884,13 @@
         <v>100</v>
       </c>
       <c r="S4" s="2" t="n">
-        <v>24.96</v>
+        <v>24.6</v>
       </c>
       <c r="T4" s="2" t="n">
         <v>25</v>
       </c>
       <c r="U4" s="2" t="n">
-        <v>12.91</v>
+        <v>13.03</v>
       </c>
       <c r="V4" s="2" t="n">
         <v>15</v>
@@ -910,12 +910,315 @@
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>2026-03-31 07:29</t>
+          <t>2026-03-31 07:47</t>
         </is>
       </c>
       <c r="AA4" s="2" t="inlineStr">
         <is>
           <t>2024-02-01 to 2026-03-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>GER40_DayTrader_v5</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Balanced</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>1H</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>USA500.IDX-USD</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>80.89</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>1450.78</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>26.97</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>61.06</v>
+      </c>
+      <c r="K5" s="2" t="n">
+        <v>53.79</v>
+      </c>
+      <c r="L5" s="2" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="M5" s="2" t="n">
+        <v>434</v>
+      </c>
+      <c r="N5" s="2" t="n">
+        <v>25.04</v>
+      </c>
+      <c r="O5" s="2" t="n">
+        <v>22.09</v>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>4/4</t>
+        </is>
+      </c>
+      <c r="Q5" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="R5" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="S5" s="2" t="n">
+        <v>15.36</v>
+      </c>
+      <c r="T5" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="U5" s="2" t="n">
+        <v>15.53</v>
+      </c>
+      <c r="V5" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="W5" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="X5" s="2" t="inlineStr">
+        <is>
+          <t>GER40_DayTrader_Strategy.pine</t>
+        </is>
+      </c>
+      <c r="Y5" s="2" t="inlineStr">
+        <is>
+          <t>ORB breakout + EMA momentum, trail 0.5 ATR</t>
+        </is>
+      </c>
+      <c r="Z5" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-31 07:47</t>
+        </is>
+      </c>
+      <c r="AA5" s="2" t="inlineStr">
+        <is>
+          <t>2024-01-01 to 2026-03-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>GER40_DayTrader_v5</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>MaxGrowth</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>1H</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>USA500.IDX-USD</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>80.13</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>2079.37</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>29.09</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>60.74</v>
+      </c>
+      <c r="K6" s="2" t="n">
+        <v>71.47</v>
+      </c>
+      <c r="L6" s="2" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="M6" s="2" t="n">
+        <v>433</v>
+      </c>
+      <c r="N6" s="2" t="n">
+        <v>37.48</v>
+      </c>
+      <c r="O6" s="2" t="n">
+        <v>33.51</v>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>4/4</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="R6" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="S6" s="2" t="n">
+        <v>14.76</v>
+      </c>
+      <c r="T6" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="U6" s="2" t="n">
+        <v>15.37</v>
+      </c>
+      <c r="V6" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="W6" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="X6" s="2" t="inlineStr">
+        <is>
+          <t>GER40_DayTrader_Strategy.pine</t>
+        </is>
+      </c>
+      <c r="Y6" s="2" t="inlineStr">
+        <is>
+          <t>ORB breakout + EMA momentum, trail 0.5 ATR</t>
+        </is>
+      </c>
+      <c r="Z6" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-31 07:47</t>
+        </is>
+      </c>
+      <c r="AA6" s="2" t="inlineStr">
+        <is>
+          <t>2024-01-01 to 2026-03-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>GER40_DayTrader_v5</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>SafeGrowth</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>1H</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>USA500.IDX-USD</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>78.66</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>574.1</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>61.5</v>
+      </c>
+      <c r="K7" s="2" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="L7" s="2" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="M7" s="2" t="n">
+        <v>439</v>
+      </c>
+      <c r="N7" s="2" t="n">
+        <v>9.779999999999999</v>
+      </c>
+      <c r="O7" s="2" t="n">
+        <v>8.83</v>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>4/4</t>
+        </is>
+      </c>
+      <c r="Q7" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="R7" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="S7" s="2" t="n">
+        <v>15.24</v>
+      </c>
+      <c r="T7" s="2" t="n">
+        <v>22.67</v>
+      </c>
+      <c r="U7" s="2" t="n">
+        <v>15.75</v>
+      </c>
+      <c r="V7" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="W7" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="X7" s="2" t="inlineStr">
+        <is>
+          <t>GER40_DayTrader_Strategy.pine</t>
+        </is>
+      </c>
+      <c r="Y7" s="2" t="inlineStr">
+        <is>
+          <t>ORB breakout + EMA momentum, trail 0.5 ATR</t>
+        </is>
+      </c>
+      <c r="Z7" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-31 07:47</t>
+        </is>
+      </c>
+      <c r="AA7" s="2" t="inlineStr">
+        <is>
+          <t>2024-01-01 to 2026-03-31</t>
         </is>
       </c>
     </row>
@@ -930,7 +1233,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1027,19 +1330,19 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>89.04000000000001</v>
+        <v>87.45999999999999</v>
       </c>
       <c r="H2" t="n">
         <v>5.43</v>
       </c>
       <c r="I2" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="J2" t="n">
-        <v>57.94</v>
+        <v>57.41</v>
       </c>
       <c r="K2" t="n">
-        <v>2.94</v>
+        <v>2.84</v>
       </c>
       <c r="L2" t="b">
         <v>1</v>
@@ -1127,19 +1430,19 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>27.22</v>
+        <v>30.45</v>
       </c>
       <c r="H4" t="n">
-        <v>4.53</v>
+        <v>4.54</v>
       </c>
       <c r="I4" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="J4" t="n">
-        <v>49.46</v>
+        <v>51.04</v>
       </c>
       <c r="K4" t="n">
-        <v>1.99</v>
+        <v>2.08</v>
       </c>
       <c r="L4" t="b">
         <v>1</v>
@@ -1177,19 +1480,19 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>41.39</v>
+        <v>40.97</v>
       </c>
       <c r="H5" t="n">
         <v>4.32</v>
       </c>
       <c r="I5" t="n">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="J5" t="n">
-        <v>53.76</v>
+        <v>54.08</v>
       </c>
       <c r="K5" t="n">
-        <v>2.6</v>
+        <v>2.52</v>
       </c>
       <c r="L5" t="b">
         <v>1</v>
@@ -1203,12 +1506,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Balanced</t>
+          <t>SafeGrowth</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>DEU.IDX-EUR</t>
+          <t>USA500.IDX-USD</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1218,28 +1521,28 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2024-02-01</t>
+          <t>2024-01-01</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2024-08-15</t>
+          <t>2024-07-23</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>138.08</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="H6" t="n">
-        <v>7.99</v>
+        <v>11.25</v>
       </c>
       <c r="I6" t="n">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="J6" t="n">
-        <v>58.49</v>
+        <v>69.61</v>
       </c>
       <c r="K6" t="n">
-        <v>2.82</v>
+        <v>2.35</v>
       </c>
       <c r="L6" t="b">
         <v>1</v>
@@ -1253,12 +1556,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Balanced</t>
+          <t>SafeGrowth</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>DEU.IDX-EUR</t>
+          <t>USA500.IDX-USD</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1268,28 +1571,28 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2024-08-16</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2025-02-28</t>
+          <t>2025-02-12</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>181.58</v>
+        <v>18.91</v>
       </c>
       <c r="H7" t="n">
-        <v>7.99</v>
+        <v>19.14</v>
       </c>
       <c r="I7" t="n">
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="J7" t="n">
-        <v>62.22</v>
+        <v>54.29</v>
       </c>
       <c r="K7" t="n">
-        <v>3.91</v>
+        <v>1.26</v>
       </c>
       <c r="L7" t="b">
         <v>1</v>
@@ -1303,12 +1606,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Balanced</t>
+          <t>SafeGrowth</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>DEU.IDX-EUR</t>
+          <t>USA500.IDX-USD</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1318,28 +1621,28 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2025-03-02</t>
+          <t>2025-02-13</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2025-09-14</t>
+          <t>2025-09-05</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>51.17</v>
+        <v>86.84999999999999</v>
       </c>
       <c r="H8" t="n">
-        <v>5.23</v>
+        <v>7.81</v>
       </c>
       <c r="I8" t="n">
-        <v>93</v>
+        <v>114</v>
       </c>
       <c r="J8" t="n">
-        <v>49.46</v>
+        <v>66.67</v>
       </c>
       <c r="K8" t="n">
-        <v>2.17</v>
+        <v>2.38</v>
       </c>
       <c r="L8" t="b">
         <v>1</v>
@@ -1353,12 +1656,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Balanced</t>
+          <t>SafeGrowth</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>DEU.IDX-EUR</t>
+          <t>USA500.IDX-USD</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1368,7 +1671,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2025-09-15</t>
+          <t>2025-09-07</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1377,19 +1680,19 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>75.47</v>
+        <v>51.41</v>
       </c>
       <c r="H9" t="n">
-        <v>5.35</v>
+        <v>20.65</v>
       </c>
       <c r="I9" t="n">
-        <v>93</v>
+        <v>118</v>
       </c>
       <c r="J9" t="n">
-        <v>53.76</v>
+        <v>55.93</v>
       </c>
       <c r="K9" t="n">
-        <v>2.85</v>
+        <v>1.57</v>
       </c>
       <c r="L9" t="b">
         <v>1</v>
@@ -1403,7 +1706,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>MaxGrowth</t>
+          <t>Balanced</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1427,19 +1730,19 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>178.54</v>
+        <v>134.92</v>
       </c>
       <c r="H10" t="n">
-        <v>8.44</v>
+        <v>7.99</v>
       </c>
       <c r="I10" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="J10" t="n">
-        <v>58.49</v>
+        <v>57.94</v>
       </c>
       <c r="K10" t="n">
-        <v>2.78</v>
+        <v>2.72</v>
       </c>
       <c r="L10" t="b">
         <v>1</v>
@@ -1453,7 +1756,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>MaxGrowth</t>
+          <t>Balanced</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1477,10 +1780,10 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>239.6</v>
+        <v>181.58</v>
       </c>
       <c r="H11" t="n">
-        <v>8.77</v>
+        <v>7.99</v>
       </c>
       <c r="I11" t="n">
         <v>90</v>
@@ -1489,7 +1792,7 @@
         <v>62.22</v>
       </c>
       <c r="K11" t="n">
-        <v>3.98</v>
+        <v>3.91</v>
       </c>
       <c r="L11" t="b">
         <v>1</v>
@@ -1503,7 +1806,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>MaxGrowth</t>
+          <t>Balanced</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1527,19 +1830,19 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>51.92</v>
+        <v>57.6</v>
       </c>
       <c r="H12" t="n">
-        <v>10.65</v>
+        <v>5.22</v>
       </c>
       <c r="I12" t="n">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="J12" t="n">
-        <v>49.46</v>
+        <v>51.04</v>
       </c>
       <c r="K12" t="n">
-        <v>1.79</v>
+        <v>2.27</v>
       </c>
       <c r="L12" t="b">
         <v>1</v>
@@ -1553,45 +1856,645 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>Balanced</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>DEU.IDX-EUR</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2025-09-15</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>74.61</v>
+      </c>
+      <c r="H13" t="n">
+        <v>5.35</v>
+      </c>
+      <c r="I13" t="n">
+        <v>98</v>
+      </c>
+      <c r="J13" t="n">
+        <v>54.08</v>
+      </c>
+      <c r="K13" t="n">
+        <v>2.74</v>
+      </c>
+      <c r="L13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>GER40_DayTrader_v5</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Balanced</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>USA500.IDX-USD</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2024-01-01</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2024-07-23</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>133.01</v>
+      </c>
+      <c r="H14" t="n">
+        <v>13.31</v>
+      </c>
+      <c r="I14" t="n">
+        <v>102</v>
+      </c>
+      <c r="J14" t="n">
+        <v>69.61</v>
+      </c>
+      <c r="K14" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="L14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>GER40_DayTrader_v5</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Balanced</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>USA500.IDX-USD</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2024-07-24</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2025-02-12</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>27.57</v>
+      </c>
+      <c r="H15" t="n">
+        <v>26.63</v>
+      </c>
+      <c r="I15" t="n">
+        <v>100</v>
+      </c>
+      <c r="J15" t="n">
+        <v>53</v>
+      </c>
+      <c r="K15" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="L15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>GER40_DayTrader_v5</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Balanced</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>USA500.IDX-USD</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2025-02-13</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2025-09-05</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>136</v>
+      </c>
+      <c r="H16" t="n">
+        <v>17.35</v>
+      </c>
+      <c r="I16" t="n">
+        <v>113</v>
+      </c>
+      <c r="J16" t="n">
+        <v>66.37</v>
+      </c>
+      <c r="K16" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="L16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>GER40_DayTrader_v5</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Balanced</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>USA500.IDX-USD</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2025-09-07</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>98.2</v>
+      </c>
+      <c r="H17" t="n">
+        <v>25.59</v>
+      </c>
+      <c r="I17" t="n">
+        <v>116</v>
+      </c>
+      <c r="J17" t="n">
+        <v>55.17</v>
+      </c>
+      <c r="K17" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="L17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>GER40_DayTrader_v5</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
           <t>MaxGrowth</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>DEU.IDX-EUR</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2024-02-01</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2024-08-15</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>174.1</v>
+      </c>
+      <c r="H18" t="n">
+        <v>10.02</v>
+      </c>
+      <c r="I18" t="n">
+        <v>107</v>
+      </c>
+      <c r="J18" t="n">
+        <v>57.94</v>
+      </c>
+      <c r="K18" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="L18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>GER40_DayTrader_v5</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>MaxGrowth</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>DEU.IDX-EUR</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2024-08-16</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2025-02-28</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>240</v>
+      </c>
+      <c r="H19" t="n">
+        <v>8.77</v>
+      </c>
+      <c r="I19" t="n">
+        <v>90</v>
+      </c>
+      <c r="J19" t="n">
+        <v>62.22</v>
+      </c>
+      <c r="K19" t="n">
+        <v>3.98</v>
+      </c>
+      <c r="L19" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>GER40_DayTrader_v5</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>MaxGrowth</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>DEU.IDX-EUR</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2025-03-02</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2025-09-14</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>60.4</v>
+      </c>
+      <c r="H20" t="n">
+        <v>10.59</v>
+      </c>
+      <c r="I20" t="n">
+        <v>96</v>
+      </c>
+      <c r="J20" t="n">
+        <v>51.04</v>
+      </c>
+      <c r="K20" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="L20" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>GER40_DayTrader_v5</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>MaxGrowth</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>DEU.IDX-EUR</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
         <is>
           <t>P4</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>2025-09-15</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>2026-03-29</t>
         </is>
       </c>
-      <c r="G13" t="n">
-        <v>102.01</v>
-      </c>
-      <c r="H13" t="n">
+      <c r="G21" t="n">
+        <v>101.3</v>
+      </c>
+      <c r="H21" t="n">
         <v>6.12</v>
       </c>
-      <c r="I13" t="n">
-        <v>93</v>
-      </c>
-      <c r="J13" t="n">
-        <v>53.76</v>
-      </c>
-      <c r="K13" t="n">
-        <v>2.93</v>
-      </c>
-      <c r="L13" t="b">
+      <c r="I21" t="n">
+        <v>98</v>
+      </c>
+      <c r="J21" t="n">
+        <v>54.08</v>
+      </c>
+      <c r="K21" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="L21" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>GER40_DayTrader_v5</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>MaxGrowth</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>USA500.IDX-USD</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2024-01-01</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2024-07-23</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>171.93</v>
+      </c>
+      <c r="H22" t="n">
+        <v>12.54</v>
+      </c>
+      <c r="I22" t="n">
+        <v>102</v>
+      </c>
+      <c r="J22" t="n">
+        <v>69.61</v>
+      </c>
+      <c r="K22" t="n">
+        <v>2.83</v>
+      </c>
+      <c r="L22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>GER40_DayTrader_v5</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>MaxGrowth</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>USA500.IDX-USD</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2024-07-24</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>2025-02-12</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>24.66</v>
+      </c>
+      <c r="H23" t="n">
+        <v>28.67</v>
+      </c>
+      <c r="I23" t="n">
+        <v>99</v>
+      </c>
+      <c r="J23" t="n">
+        <v>52.53</v>
+      </c>
+      <c r="K23" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="L23" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>GER40_DayTrader_v5</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>MaxGrowth</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>USA500.IDX-USD</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2025-02-13</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2025-09-05</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>165.22</v>
+      </c>
+      <c r="H24" t="n">
+        <v>20.03</v>
+      </c>
+      <c r="I24" t="n">
+        <v>113</v>
+      </c>
+      <c r="J24" t="n">
+        <v>65.48999999999999</v>
+      </c>
+      <c r="K24" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="L24" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>GER40_DayTrader_v5</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>MaxGrowth</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>USA500.IDX-USD</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2025-09-07</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>118.72</v>
+      </c>
+      <c r="H25" t="n">
+        <v>27.65</v>
+      </c>
+      <c r="I25" t="n">
+        <v>116</v>
+      </c>
+      <c r="J25" t="n">
+        <v>55.17</v>
+      </c>
+      <c r="K25" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="L25" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>